<commit_message>
Add redemption toggle to /model and refresh workbook
</commit_message>
<xml_diff>
--- a/model/TGP_Fund_One_Model.xlsx
+++ b/model/TGP_Fund_One_Model.xlsx
@@ -153,7 +153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -276,6 +276,11 @@
       <c r="B11" s="5">
         <v>0.0</v>
       </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t>Web model settings reference</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="3">
@@ -286,6 +291,16 @@
       <c r="B12" s="6">
         <v>0.25</v>
       </c>
+      <c r="C12" t="inlineStr" s="3">
+        <is>
+          <t>Redemptions On</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="10">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="3">
@@ -296,6 +311,16 @@
       <c r="B13" s="6">
         <v>0.18</v>
       </c>
+      <c r="C13" t="inlineStr" s="3">
+        <is>
+          <t>Lockup (months)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="10">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="3">
@@ -306,6 +331,16 @@
       <c r="B14" s="6">
         <v>0.08</v>
       </c>
+      <c r="C14" t="inlineStr" s="3">
+        <is>
+          <t>Liquidity Event (months)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="10">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="3">
@@ -316,6 +351,16 @@
       <c r="B15" s="6">
         <v>0.15</v>
       </c>
+      <c r="C15" t="inlineStr" s="3">
+        <is>
+          <t>Liquidity Request</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="10">
+        <is>
+          <t>5.0%</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="3">
@@ -326,6 +371,28 @@
       <c r="B16" s="5">
         <v>120</v>
       </c>
+      <c r="C16" t="inlineStr" s="3">
+        <is>
+          <t>Switch Rate</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="10">
+        <is>
+          <t>25.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr" s="3">
+        <is>
+          <t>Cash Payout Cap</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="10">
+        <is>
+          <t>5.0%</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="2">
@@ -333,6 +400,16 @@
           <t>Derived</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr" s="3">
+        <is>
+          <t>GP Hurdle</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="10">
+        <is>
+          <t>8.0%</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="3">
@@ -342,6 +419,16 @@
       </c>
       <c r="B19" s="5">
         <f>IF(B7=1,0,B6)</f>
+      </c>
+      <c r="C19" t="inlineStr" s="3">
+        <is>
+          <t>GP Carry</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="10">
+        <is>
+          <t>15.0%</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -497,6 +584,11 @@
       </c>
       <c r="B10" s="7">
         <f>MAX(Monthly_Model!$V$8:$V$127)</f>
+      </c>
+      <c r="C10" t="inlineStr" s="10">
+        <is>
+          <t>The live /model page also includes redemption toggles, liquidity windows, GP carry units, and investor liquidity readouts.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -14350,7 +14442,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
@@ -14421,22 +14513,46 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="3">
         <is>
-          <t>How origination scales</t>
+          <t>Redemptions</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="10">
         <is>
-          <t>Desired origination volume is driven by pipeline capacity and deployable capital. In normal mode the model ramps scaling over 12 months. Hardcore Mode removes that gentler ramp and pushes available cash out immediately.</t>
+          <t>The live web model can toggle redemptions on or off and layer lockup, liquidity windows, switch rates, and cash payout caps on top of the core origination model.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="3">
         <is>
+          <t>GP units</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="10">
+        <is>
+          <t>The live web model also mints GP units above the hurdle and tracks GP ownership dilution over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="3">
+        <is>
+          <t>How origination scales</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="10">
+        <is>
+          <t>Desired origination volume is driven by pipeline capacity and deployable capital. In normal mode the model ramps scaling over 12 months. Hardcore Mode removes that gentler ramp and pushes available cash out immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="3">
+        <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="10">
+      <c r="B11" t="inlineStr" s="10">
         <is>
           <t>Projected IRR is solved from LP cash calls and terminal NAV. The Monthly_Model sheet also includes an IRR To Date column.</t>
         </is>

</xml_diff>